<commit_message>
Reconciliation: second self-check (psych status, link to 13.10 reconciliation, admission risk)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018E5oU3tu1dsgPCGBpryD3s
</commit_message>
<xml_diff>
--- a/Сверка_МО_со_штаткой_05.10.2026.xlsx
+++ b/Сверка_МО_со_штаткой_05.10.2026.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="264">
   <si>
     <t xml:space="preserve">Сверка списка медосмотров со штатным расписанием</t>
   </si>
@@ -74,13 +74,13 @@
     <t xml:space="preserve">1. Уволены 6 чел. (Воронеж 1, Машково 1, Руднево 4). У 4 из них в файле стоит дата предварительного МО — исторические данные можно сохранить в архиве, из действующего списка исключить.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Принято 10 чел. на должности из перечня (08.09–02.10.2026). Даты предварительного МО по ним в файле нет — проверить, что осмотр пройден ДО допуска к работе (ст. 214, 220 ТК РФ). Власова О.В. (электромонтажник, п.20) — дополнительно психиатрическое освидетельствование. У Иванова Ю.С. в штатке не указано фактическое место работы.</t>
+    <t xml:space="preserve">2. Принято 10 чел. на должности из перечня (08.09–02.10.2026). Даты предварительного МО по ним в файле нет — проверить, что осмотр пройден ДО допуска к работе (ст. 214, 220 ТК РФ). Власова О.В. (электромонтажник, п.20): психиатрическое освидетельствование — «Проверить» (см. слабые места, п.5). У Иванова Ю.С. в штатке не указано фактическое место работы.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Главный риск: 33 чел. мебельного участка и участка декоративной отделки (Машково) в штатке переименованы — «Столяр», «Столяр-краснодеревщик» → «Техник-сборщик»; «Маляр» → «Техник»; «Оператор-наладчик станков с ЧПУ» → «Инженер-программист станков с ЧПУ». Этих наименований нет в Приказе №43. Обязанность МО определяется вредными факторами и видами работ (Приказ №29н, ст. 220 ТК РФ), а не названием должности: работа с ЛКМ, древесной пылью, шумом сохраняется. Исключать их из списка нельзя — нужно внести изменения в Приказ №43 и уточнить у кадровой службы основание переименования.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Монтажники электрооборудования ЛА (4 чел., Машково) переведены в «Электромонтажник» (п.20) — у них появляется обязанность психиатрического освидетельствования (п.20 = «Да»).</t>
+    <t xml:space="preserve">4. Монтажники электрооборудования ЛА (4 чел., Машково) переведены в «Электромонтажник» (п.20). По п.20 нет химических факторов п.37 (1.8.4, 1.12, 1.15, 1.25, 1.27, 1.44, 4.6) — если работа прежняя, объём осмотра сокращается неправомерно. Психиатрическое освидетельствование: п.11 Прил.№2 к 342н касается электроустановок «в сфере электроэнергетики»; применимость к монтажу бортового ЭО спорна — статус «Проверить», решение работодателя с обоснованием.</t>
   </si>
   <si>
     <t xml:space="preserve">5. «Оператор станков с ЧПУ» (штатка) vs «Оператор станка с ЧПУ» (Приказ №43, п.30) — разночтение в написании. Отнесены к п.30; в Приказе №43 при следующей редакции привести формулировку к штатке. В лист «Соответствие» добавить ключ «оператор станков с чпу» → 30.</t>
@@ -122,6 +122,24 @@
     <t xml:space="preserve">9. Анисимов И.В. (сборщик стеклопластиковых изделий) — 20,9 года. Периодичность 12 мес. совпадает с правилом для лиц моложе 21 года, отдельных действий не требуется.</t>
   </si>
   <si>
+    <t xml:space="preserve">Самопроверка №2 (15.10.2026): что найдено дополнительно</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. ДУБЛИРОВАНИЕ. В репозитории уже есть сверка с той же штаткой от 13.10.2026 — «Медосмотры_сверка_штатка_05.10.2026.xlsx» (учёт обновлён до 371 чел., лист «Выбывшие», раздел требований 7.1–7.21) и «Проект изменений в приказ 43» (позиции №46 «Техник-сборщик», №47 «Техник», п.30 «станка/станков»). Загруженный для сверки файл МО — версия от 10.09.2026, до этих изменений. Рабочим (мастер-) файлом следует считать файл от 13.10.2026; настоящий отчёт — независимая перекрёстная проверка.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Результаты совпали с файлом от 13.10 по всем ключевым цифрам: 6 уволенных (те же ФИО), 33 переименования вне перечня, 14 переводов со сменой пунктов, 11 должностей на оценку по СОУТ. Расхождение: Кляцкин А.Б. и Каретников Р.Г. в файле от 13.10 добавлены в учёт (12 новых, по будущим позициям №46/47), здесь — на листе 4 (10 новых). С учётом проекта изменений правильнее 12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12. Пропущено в первой версии отчёта: из принятых после 03.04.2026 (40 чел. в старом файле МО + 12 новых, за вычетом 3 уволенных = 49) у 33 нет даты предварительного МО. Если осмотр фактически не проводился — это допуск к работе без обязательного медосмотра: обязанность отстранить (ст. 76 ТК РФ), штраф для юрлица 110–130 тыс. руб. за каждого работника (ч.3 ст. 5.27.1 КоАП РФ). Это самый срочный пункт — запросить заключения в медорганизации.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13. Проект изменений в приказ №43 проверен по штатке 05.10: Будавских В.Г. (мастер участка сборки интерьера), Жусев А.А. (инженер-электрик), Рукин Д.И. (старший охраны объекта), Климачев С.В. (зам. директора департамента — нач. ПП), 14 чел. ОТК, 21 чел. ПДО (+2 диспетчера Казань), 9 водителей-экспедиторов, 22 техника-сборщика, 12 техников, 4 оператора «станков с ЧПУ» — подтверждено. До подписания: заполнить «п.18.__.» по позиции №38 (категории ТС у 9 водителей); решить вопрос по 4 бывшим монтажникам ЭО ЛА.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14. Ошибка первой версии отчёта исправлена: психиатрическое освидетельствование для п.20/п.29 указывалось «Да». Исправлено на «Проверить» (листы 2, 3, вывод 4).</t>
+  </si>
+  <si>
     <t xml:space="preserve">№</t>
   </si>
   <si>
@@ -278,7 +296,7 @@
     <t xml:space="preserve">Электромонтажник</t>
   </si>
   <si>
-    <t xml:space="preserve">Да</t>
+    <t xml:space="preserve">Проверить</t>
   </si>
   <si>
     <t xml:space="preserve">Ефременко Роман Вадимович</t>
@@ -575,7 +593,7 @@
     <t xml:space="preserve">Электромонтажник 5 разряда</t>
   </si>
   <si>
-    <t xml:space="preserve">Другой пункт — обновить должность и пункт; меняется статус психиатр. освид.</t>
+    <t xml:space="preserve">Другой пункт — обновить должность и пункт; психиатр. освид. — проверить применимость п.11 Прил.2 342н</t>
   </si>
   <si>
     <t xml:space="preserve">п.1.8.4, п.1.12, п.1.15, п.1.25, п.1.27, п.1.44, п.4.6</t>
@@ -954,7 +972,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -985,6 +1003,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1332,7 +1354,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="80"/>
@@ -1447,7 +1469,7 @@
       </c>
       <c r="B15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>14</v>
       </c>
@@ -1459,7 +1481,7 @@
       </c>
       <c r="B17" s="4"/>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
         <v>16</v>
       </c>
@@ -1483,7 +1505,7 @@
       </c>
       <c r="B21" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
         <v>20</v>
       </c>
@@ -1542,8 +1564,43 @@
       </c>
       <c r="B32" s="4"/>
     </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="22">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A16:B16"/>
@@ -1561,6 +1618,11 @@
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1591,32 +1653,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>38</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1627,23 +1689,23 @@
         <v>53</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="G2" s="11" t="n">
         <v>45770</v>
       </c>
       <c r="H2" s="6"/>
-      <c r="I2" s="11" t="s">
-        <v>43</v>
+      <c r="I2" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1654,25 +1716,25 @@
         <v>99</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="G3" s="11" t="n">
         <v>46139</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="11" t="n">
         <v>46127</v>
       </c>
-      <c r="I3" s="11" t="s">
-        <v>43</v>
+      <c r="I3" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1683,25 +1745,25 @@
         <v>303</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>46140</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>46134</v>
+      </c>
+      <c r="I4" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>46140</v>
-      </c>
-      <c r="H4" s="10" t="n">
-        <v>46134</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1712,23 +1774,23 @@
         <v>305</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="G5" s="11" t="n">
         <v>46036</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="I5" s="11" t="s">
-        <v>43</v>
+      <c r="I5" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1739,25 +1801,25 @@
         <v>319</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <v>45950</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="11" t="n">
         <v>45941</v>
       </c>
-      <c r="I6" s="11" t="s">
-        <v>43</v>
+      <c r="I6" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1768,25 +1830,25 @@
         <v>323</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>46156</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="11" t="n">
         <v>46147</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>43</v>
+      <c r="I7" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1823,41 +1885,41 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="L1" s="9" t="s">
+      <c r="B1" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>64</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1865,324 +1927,324 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F2" s="10" t="n">
+        <v>74</v>
+      </c>
+      <c r="F2" s="11" t="n">
         <v>46286</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>30</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" s="11" t="n">
         <v>46269</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>14</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J3" s="6"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F4" s="11" t="n">
         <v>46286</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>19</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J4" s="6"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F5" s="11" t="n">
         <v>46293</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J5" s="6"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F6" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F6" s="11" t="n">
         <v>46296</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>19</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F7" s="11" t="n">
         <v>46286</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>26</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J7" s="6"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <v>46290</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>18</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J8" s="6"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F9" s="11" t="n">
         <v>46296</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>30</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="F10" s="11" t="n">
         <v>46296</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>11</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J10" s="6"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="F11" s="11" t="n">
         <v>46297</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>14</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J11" s="6"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L11"/>
@@ -2215,51 +2277,51 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="K1" s="9" t="s">
+      <c r="A1" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="H1" s="10" t="s">
         <v>107</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2270,38 +2332,38 @@
         <v>137</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="H2" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L2" s="6"/>
-      <c r="M2" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>113</v>
+      <c r="M2" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2312,38 +2374,38 @@
         <v>138</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L3" s="6"/>
-      <c r="M3" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N3" s="11" t="s">
-        <v>113</v>
+      <c r="M3" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N3" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2354,38 +2416,38 @@
         <v>139</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="H4" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L4" s="6"/>
-      <c r="M4" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>113</v>
+      <c r="M4" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2396,38 +2458,38 @@
         <v>140</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L5" s="6"/>
-      <c r="M5" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>113</v>
+      <c r="M5" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N5" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2438,38 +2500,38 @@
         <v>142</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L6" s="6"/>
-      <c r="M6" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>113</v>
+      <c r="M6" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N6" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2480,38 +2542,38 @@
         <v>147</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L7" s="6"/>
-      <c r="M7" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>124</v>
+      <c r="M7" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2522,38 +2584,38 @@
         <v>148</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L8" s="6"/>
-      <c r="M8" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>124</v>
+      <c r="M8" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2564,38 +2626,38 @@
         <v>149</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L9" s="6"/>
-      <c r="M9" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>124</v>
+      <c r="M9" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N9" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2606,38 +2668,38 @@
         <v>150</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L10" s="6"/>
-      <c r="M10" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>124</v>
+      <c r="M10" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2648,38 +2710,38 @@
         <v>151</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>122</v>
-      </c>
       <c r="G11" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L11" s="6"/>
-      <c r="M11" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N11" s="11" t="s">
-        <v>124</v>
+      <c r="M11" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,38 +2752,38 @@
         <v>152</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L12" s="6"/>
-      <c r="M12" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N12" s="11" t="s">
-        <v>124</v>
+      <c r="M12" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2732,38 +2794,38 @@
         <v>153</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L13" s="6"/>
-      <c r="M13" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>124</v>
+      <c r="M13" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2774,38 +2836,38 @@
         <v>154</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>24</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L14" s="6"/>
-      <c r="M14" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>124</v>
+      <c r="M14" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N14" s="12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2816,38 +2878,38 @@
         <v>155</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L15" s="6"/>
-      <c r="M15" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N15" s="11" t="s">
-        <v>113</v>
+      <c r="M15" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N15" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2858,38 +2920,38 @@
         <v>156</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L16" s="6"/>
-      <c r="M16" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N16" s="11" t="s">
-        <v>113</v>
+      <c r="M16" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N16" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2900,38 +2962,38 @@
         <v>157</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L17" s="6"/>
-      <c r="M17" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>113</v>
+      <c r="M17" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N17" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2942,38 +3004,38 @@
         <v>158</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L18" s="6"/>
-      <c r="M18" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>113</v>
+      <c r="M18" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N18" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2984,38 +3046,38 @@
         <v>159</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L19" s="6"/>
-      <c r="M19" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N19" s="11" t="s">
-        <v>113</v>
+      <c r="M19" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N19" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3026,38 +3088,38 @@
         <v>160</v>
       </c>
       <c r="C20" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F20" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="G20" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L20" s="6"/>
-      <c r="M20" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N20" s="11" t="s">
-        <v>113</v>
+      <c r="M20" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N20" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3068,38 +3130,38 @@
         <v>162</v>
       </c>
       <c r="C21" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L21" s="6"/>
-      <c r="M21" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N21" s="11" t="s">
-        <v>113</v>
+      <c r="M21" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N21" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3110,38 +3172,38 @@
         <v>171</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>25</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L22" s="6"/>
-      <c r="M22" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N22" s="11" t="s">
-        <v>144</v>
+      <c r="M22" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N22" s="12" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3152,40 +3214,40 @@
         <v>177</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>21</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L23" s="10" t="n">
+        <v>117</v>
+      </c>
+      <c r="L23" s="11" t="n">
         <v>46171</v>
       </c>
-      <c r="M23" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N23" s="11" t="s">
-        <v>113</v>
+      <c r="M23" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N23" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3196,38 +3258,38 @@
         <v>183</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L24" s="6"/>
-      <c r="M24" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N24" s="11" t="s">
-        <v>152</v>
+      <c r="M24" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3238,38 +3300,38 @@
         <v>188</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L25" s="6"/>
-      <c r="M25" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N25" s="11" t="s">
-        <v>152</v>
+      <c r="M25" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N25" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3280,38 +3342,38 @@
         <v>189</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>157</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="H26" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L26" s="6"/>
-      <c r="M26" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N26" s="11" t="s">
-        <v>152</v>
+      <c r="M26" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N26" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3322,38 +3384,38 @@
         <v>190</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E27" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G27" s="6" t="s">
         <v>157</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L27" s="6"/>
-      <c r="M27" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N27" s="11" t="s">
-        <v>152</v>
+      <c r="M27" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3364,38 +3426,38 @@
         <v>191</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E28" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>157</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L28" s="6"/>
-      <c r="M28" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N28" s="11" t="s">
-        <v>152</v>
+      <c r="M28" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N28" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3406,38 +3468,38 @@
         <v>192</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H29" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L29" s="6"/>
-      <c r="M29" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N29" s="11" t="s">
-        <v>152</v>
+      <c r="M29" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N29" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3448,38 +3510,38 @@
         <v>193</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L30" s="6"/>
-      <c r="M30" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N30" s="11" t="s">
-        <v>152</v>
+      <c r="M30" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N30" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3490,40 +3552,40 @@
         <v>194</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H31" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L31" s="10" t="n">
+        <v>117</v>
+      </c>
+      <c r="L31" s="11" t="n">
         <v>46157</v>
       </c>
-      <c r="M31" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N31" s="11" t="s">
-        <v>152</v>
+      <c r="M31" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N31" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3534,38 +3596,38 @@
         <v>195</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H32" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L32" s="6"/>
-      <c r="M32" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N32" s="11" t="s">
-        <v>152</v>
+      <c r="M32" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N32" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3576,40 +3638,40 @@
         <v>196</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H33" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L33" s="10" t="n">
+        <v>117</v>
+      </c>
+      <c r="L33" s="11" t="n">
         <v>46220</v>
       </c>
-      <c r="M33" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N33" s="11" t="s">
-        <v>152</v>
+      <c r="M33" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N33" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3620,38 +3682,38 @@
         <v>197</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H34" s="6" t="n">
         <v>36</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="L34" s="6"/>
-      <c r="M34" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N34" s="11" t="s">
-        <v>152</v>
+      <c r="M34" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N34" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,19 +3724,19 @@
         <v>84</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>18</v>
@@ -3683,17 +3745,17 @@
         <v>18</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L35" s="6"/>
-      <c r="M35" s="13" t="s">
-        <v>174</v>
+      <c r="M35" s="14" t="s">
+        <v>180</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3704,19 +3766,19 @@
         <v>85</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H36" s="6" t="n">
         <v>18</v>
@@ -3725,19 +3787,19 @@
         <v>18</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="L36" s="10" t="n">
+        <v>76</v>
+      </c>
+      <c r="L36" s="11" t="n">
         <v>45825</v>
       </c>
-      <c r="M36" s="13" t="s">
-        <v>174</v>
+      <c r="M36" s="14" t="s">
+        <v>180</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3748,19 +3810,19 @@
         <v>86</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H37" s="6" t="n">
         <v>18</v>
@@ -3769,17 +3831,17 @@
         <v>18</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L37" s="6"/>
-      <c r="M37" s="13" t="s">
-        <v>174</v>
+      <c r="M37" s="14" t="s">
+        <v>180</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3790,19 +3852,19 @@
         <v>133</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H38" s="6" t="n">
         <v>37</v>
@@ -3811,19 +3873,19 @@
         <v>20</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="L38" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="L38" s="11" t="n">
         <v>45840</v>
       </c>
-      <c r="M38" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="N38" s="11" t="s">
-        <v>182</v>
+      <c r="M38" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="N38" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3834,19 +3896,19 @@
         <v>134</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H39" s="6" t="n">
         <v>37</v>
@@ -3855,17 +3917,17 @@
         <v>20</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="L39" s="6"/>
-      <c r="M39" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="N39" s="11" t="s">
-        <v>182</v>
+      <c r="M39" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="N39" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3876,19 +3938,19 @@
         <v>135</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E40" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F40" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>179</v>
-      </c>
       <c r="G40" s="6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H40" s="6" t="n">
         <v>37</v>
@@ -3897,17 +3959,17 @@
         <v>20</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="L40" s="6"/>
-      <c r="M40" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="N40" s="11" t="s">
-        <v>182</v>
+      <c r="M40" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="N40" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3918,19 +3980,19 @@
         <v>136</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G41" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>180</v>
       </c>
       <c r="H41" s="6" t="n">
         <v>37</v>
@@ -3939,17 +4001,17 @@
         <v>20</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="L41" s="6"/>
-      <c r="M41" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="N41" s="11" t="s">
-        <v>182</v>
+      <c r="M41" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="N41" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3960,19 +4022,19 @@
         <v>143</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H42" s="6" t="n">
         <v>30</v>
@@ -3981,17 +4043,17 @@
         <v>30</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L42" s="6"/>
-      <c r="M42" s="13" t="s">
-        <v>188</v>
+      <c r="M42" s="14" t="s">
+        <v>194</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4002,19 +4064,19 @@
         <v>146</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="H43" s="6" t="n">
         <v>30</v>
@@ -4023,17 +4085,17 @@
         <v>30</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L43" s="6"/>
-      <c r="M43" s="13" t="s">
-        <v>188</v>
+      <c r="M43" s="14" t="s">
+        <v>194</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4044,19 +4106,19 @@
         <v>161</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H44" s="6" t="n">
         <v>21</v>
@@ -4065,17 +4127,17 @@
         <v>18</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L44" s="6"/>
-      <c r="M44" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N44" s="11" t="s">
-        <v>195</v>
+      <c r="M44" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N44" s="12" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4086,19 +4148,19 @@
         <v>164</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H45" s="6" t="n">
         <v>26</v>
@@ -4107,17 +4169,17 @@
         <v>18</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L45" s="6"/>
-      <c r="M45" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N45" s="11" t="s">
-        <v>198</v>
+      <c r="M45" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N45" s="12" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4128,19 +4190,19 @@
         <v>174</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>26</v>
@@ -4149,17 +4211,17 @@
         <v>23</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L46" s="6"/>
-      <c r="M46" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N46" s="11" t="s">
-        <v>202</v>
+      <c r="M46" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N46" s="12" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4170,19 +4232,19 @@
         <v>179</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>36</v>
@@ -4191,17 +4253,17 @@
         <v>18</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L47" s="6"/>
-      <c r="M47" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N47" s="11" t="s">
-        <v>204</v>
+      <c r="M47" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N47" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4212,19 +4274,19 @@
         <v>180</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>36</v>
@@ -4233,17 +4295,17 @@
         <v>18</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L48" s="6"/>
-      <c r="M48" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N48" s="11" t="s">
-        <v>204</v>
+      <c r="M48" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N48" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4254,19 +4316,19 @@
         <v>181</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H49" s="6" t="n">
         <v>36</v>
@@ -4275,17 +4337,17 @@
         <v>23</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L49" s="6"/>
-      <c r="M49" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N49" s="11" t="s">
-        <v>208</v>
+      <c r="M49" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N49" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4296,19 +4358,19 @@
         <v>182</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H50" s="6" t="n">
         <v>36</v>
@@ -4317,17 +4379,17 @@
         <v>23</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L50" s="6"/>
-      <c r="M50" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N50" s="11" t="s">
-        <v>208</v>
+      <c r="M50" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N50" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4338,19 +4400,19 @@
         <v>185</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="H51" s="6" t="n">
         <v>36</v>
@@ -4359,17 +4421,17 @@
         <v>23</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L51" s="6"/>
-      <c r="M51" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N51" s="11" t="s">
-        <v>208</v>
+      <c r="M51" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N51" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4380,19 +4442,19 @@
         <v>321</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="H52" s="6" t="n">
         <v>43</v>
@@ -4401,19 +4463,19 @@
         <v>32</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="L52" s="10" t="n">
+        <v>76</v>
+      </c>
+      <c r="L52" s="11" t="n">
         <v>45922</v>
       </c>
-      <c r="M52" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N52" s="11" t="s">
-        <v>216</v>
+      <c r="M52" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N52" s="12" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4424,19 +4486,19 @@
         <v>322</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="H53" s="6" t="n">
         <v>43</v>
@@ -4445,19 +4507,19 @@
         <v>32</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="L53" s="10" t="n">
+        <v>76</v>
+      </c>
+      <c r="L53" s="11" t="n">
         <v>45926</v>
       </c>
-      <c r="M53" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="N53" s="11" t="s">
-        <v>216</v>
+      <c r="M53" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="N53" s="12" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -4492,45 +4554,45 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="A1" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>223</v>
+      <c r="B2" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4538,324 +4600,324 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F3" s="11" t="n">
         <v>46267</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I3" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F4" s="11" t="n">
         <v>46163</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I4" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F5" s="11" t="n">
         <v>40210</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I5" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>44258</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>44258</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I6" s="12"/>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F7" s="11" t="n">
         <v>40878</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I7" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <v>46286</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I8" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="F9" s="11" t="n">
         <v>45028</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I9" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="F10" s="11" t="n">
         <v>46237</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I10" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="10" t="n">
+        <v>57</v>
+      </c>
+      <c r="F11" s="11" t="n">
         <v>46286</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I11" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>42461</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I12" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F13" s="11" t="n">
         <v>45180</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I13" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F14" s="11" t="n">
         <v>40030</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I14" s="12"/>
+        <v>232</v>
+      </c>
+      <c r="I14" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:I14"/>

</xml_diff>